<commit_message>
chore(): add more AE/BE terms
</commit_message>
<xml_diff>
--- a/BE_AE.xlsx
+++ b/BE_AE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B187"/>
+  <dimension ref="A1:B365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2660,6 +2660,2142 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>colours</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>colors</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>coloured</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>colored</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>colouring</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>coloring</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>colourful</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>colorful</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>colourless</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>colorless</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>honours</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>honors</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>honoured</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>honored</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>honouring</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>honoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>honourable</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>honorable</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>favours</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>favors</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>favoured</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>favored</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>favouring</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>favoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>favourite</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>favorite</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>favourites</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>favorites</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>favourable</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>favorable</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>favourably</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>favorably</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>neighbours</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>neighbors</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>neighbouring</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>neighboring</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>neighbourhood</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>neighborhood</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>neighbourhoods</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>neighborhoods</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>behaviours</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>behaviors</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>behavioural</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>behavioral</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>behaviourally</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>behaviorally</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>harbours</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>harbors</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>harboured</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>harbored</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>harbouring</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>harboring</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>laboured</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>labored</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>labouring</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>laboring</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>labours</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>labors</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>labourer</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>laborer</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>labourers</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>laborers</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>odours</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>odors</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>odourless</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>odorless</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>rumours</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>rumors</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>rumoured</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>rumored</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>vapours</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>vapors</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>vapourise</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>vaporize</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>vapourised</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>vaporized</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>armoured</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>armored</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>armours</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>armors</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>endeavours</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>endeavors</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>endeavoured</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>endeavored</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>endeavouring</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>endeavoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>savours</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>savors</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>savoured</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>savored</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>savouring</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>savoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>savoury</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>savory</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>flavours</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>flavors</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>flavoured</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>flavored</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>flavouring</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>flavoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>flavourful</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>flavorful</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>realised</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>realized</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>realising</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>realizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>realises</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>realizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>realisation</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>realization</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>realisations</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>realizations</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>recognised</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>recognized</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>recognising</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>recognizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>recognises</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>recognizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>recognisable</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>recognizable</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>organised</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>organized</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>organising</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>organizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>organises</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>organizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>organisation</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>organisations</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>organizations</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>organiser</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>organisers</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>organizers</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>emphasised</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>emphasized</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>emphasising</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>emphasizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>emphasises</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>emphasizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>analysed</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>analyzed</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>analysing</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>analyzing</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>apologised</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>apologized</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>apologising</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>apologizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>apologises</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>apologizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>criticised</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>criticized</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>criticising</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>criticizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>criticises</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>criticizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>memorised</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>memorized</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>memorising</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>memorizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>memorises</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>memorizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>specialised</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>specialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>specialising</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>specializing</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>specialises</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>specializes</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>specialisation</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>specialization</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>summarised</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>summarized</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>summarising</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>summarizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>summarises</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>summarizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>utilised</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>utilized</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>utilising</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>utilizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>utilises</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>utilizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>utilisation</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>utilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>visualised</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>visualized</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>visualising</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>visualizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>visualises</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>visualizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>visualisation</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>visualization</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>materialised</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>materialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>materialising</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>materializing</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>materialises</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>materializes</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>materialisation</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>materialization</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>symbolised</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>symbolized</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>symbolising</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>symbolizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>symbolises</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>symbolizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>symbolisation</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>symbolization</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>harmonised</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>harmonized</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>harmonising</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>harmonizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>harmonises</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>harmonizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>harmonisation</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>harmonization</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>characterised</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>characterized</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>characterising</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>characterizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>characterises</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>characterizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>characterisation</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>characterization</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>arbour</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>arbor</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>candour</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>candor</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>demeanour</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>demeanor</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>fervour</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>fervor</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>parlour</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>parlor</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>rancour</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>rancor</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>rigour</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>rigor</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>rigours</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>rigors</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>succour</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>succor</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>tumour</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>tumor</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>tumours</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>tumors</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>valour</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>ardour</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>ardor</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>glamour</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>glamor</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>baptise</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>baptize</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>baptised</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>baptized</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>baptising</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>baptizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>baptises</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>baptizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>evangelise</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>evangelize</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>evangelised</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>evangelized</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>evangelising</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>evangelizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>evangelises</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>evangelizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>hospitalise</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>hospitalize</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>hospitalised</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>hospitalized</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>hospitalising</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>hospitalizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>prioritise</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>prioritize</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>prioritised</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>prioritized</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>prioritising</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>prioritizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>prioritises</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>prioritizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>patronise</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>patronize</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>patronised</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>patronized</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>patronising</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>patronizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>patronises</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>patronizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>antagonise</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>antagonize</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>antagonised</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>antagonized</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>antagonising</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>antagonizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>antagonises</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>antagonizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>sympathise</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>sympathize</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>sympathised</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>sympathized</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>sympathising</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>sympathizing</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>sympathises</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>sympathizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>paralyse</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>paralyze</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>paralysed</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>paralyzed</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>paralysing</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>paralyzing</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>aluminium</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>aluminum</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>moustache</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>mustache</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>dialogue</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>dialog</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>dialogues</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>dialogs</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>spelt</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>spelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>learnt</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>dreamt</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>dreamed</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>leapt</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>leaped</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>spoilt</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>spoiled</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>worshipping</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>worshiping</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>worshipped</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>worshiped</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>worshipper</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>worshiper</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>worshippers</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>worshipers</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>dialled</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>dialed</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>dialling</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>dialing</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>focussed</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>focused</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>focussing</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>focusing</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>focusses</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>focuses</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>equalled</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>equaled</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>equalling</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>equaling</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>levelled</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>leveled</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>levelling</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>leveling</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>